<commit_message>
Write A440 to WAV File
Created Java project wavwriter with method main to write ten seconds of A440 to A440.wav.
</commit_message>
<xml_diff>
--- a/Interface_Design/System_Interface_Design.xlsx
+++ b/Interface_Design/System_Interface_Design.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="23628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="23801"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thoma\Documents\GitHub\Audio_Analyzer\Interface_Design\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{076D12DD-43E8-4CF4-B8D8-5F9C2CB1F58E}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0442E541-2C6D-4A96-9294-FE20D69F4846}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19320" yWindow="100" windowWidth="18920" windowHeight="20770" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="140" yWindow="20" windowWidth="19140" windowHeight="20780" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>